<commit_message>
continue data gathering scenarios
</commit_message>
<xml_diff>
--- a/Documents/DBdesign.xlsx
+++ b/Documents/DBdesign.xlsx
@@ -1,36 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E01B8D-64A9-47F1-86BA-ABA48CF1A353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF10D9F-43C9-40F4-8D65-AD815682AEAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BEC21941-B947-480A-A7E6-7B63159DE119}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="2" xr2:uid="{BEC21941-B947-480A-A7E6-7B63159DE119}"/>
   </bookViews>
   <sheets>
     <sheet name="RBAC+ABAC" sheetId="1" r:id="rId1"/>
-    <sheet name="Candidate" sheetId="2" r:id="rId2"/>
+    <sheet name="MSForms" sheetId="2" r:id="rId2"/>
+    <sheet name="Company Setup" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
@@ -40,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="92">
   <si>
     <t>JobOfferUsers</t>
   </si>
@@ -243,24 +233,9 @@
     <t>CandidateApplications</t>
   </si>
   <si>
-    <t>HiringCompanyId</t>
-  </si>
-  <si>
-    <t>ApplicationStatusId</t>
-  </si>
-  <si>
     <t>CurrentWorkflowStatusId</t>
   </si>
   <si>
-    <t>ApplicationDate</t>
-  </si>
-  <si>
-    <t>EndorsementDate</t>
-  </si>
-  <si>
-    <t>TAOwnerId</t>
-  </si>
-  <si>
     <t>RequestSentDate</t>
   </si>
   <si>
@@ -286,6 +261,51 @@
   </si>
   <si>
     <t>ReferenceNumber</t>
+  </si>
+  <si>
+    <t>FileName</t>
+  </si>
+  <si>
+    <t>FilePath</t>
+  </si>
+  <si>
+    <t>FileSize</t>
+  </si>
+  <si>
+    <t>FileTypeId</t>
+  </si>
+  <si>
+    <t>UploadedBy</t>
+  </si>
+  <si>
+    <t>UploadedDate</t>
+  </si>
+  <si>
+    <t>FileTypes</t>
+  </si>
+  <si>
+    <t>TypeName</t>
+  </si>
+  <si>
+    <t>SubmittedDocuments</t>
+  </si>
+  <si>
+    <t>CurrencyId</t>
+  </si>
+  <si>
+    <t>Currencies</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>CreatedBy</t>
+  </si>
+  <si>
+    <t>CreatedAt</t>
   </si>
 </sst>
 </file>
@@ -991,15 +1011,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{026B99F0-FC57-47AB-AF03-F4ABCCD02BF2}">
-  <dimension ref="B2:F16"/>
+  <dimension ref="B2:H16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="22.54296875" customWidth="1"/>
-    <col min="4" max="4" width="23.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
         <v>53</v>
       </c>
@@ -1007,10 +1027,13 @@
         <v>65</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+        <v>85</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>1</v>
       </c>
@@ -1020,8 +1043,11 @@
       <c r="F3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="H3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>54</v>
       </c>
@@ -1031,110 +1057,179 @@
       <c r="F4" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="H4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>55</v>
       </c>
       <c r="D5" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>56</v>
       </c>
       <c r="D6" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F6" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>57</v>
       </c>
       <c r="D8" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F8" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>58</v>
       </c>
       <c r="D9" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F10" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>60</v>
       </c>
       <c r="D11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="F11" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AD6FEA5-0945-4178-A2F8-A72772503D4A}">
+  <dimension ref="B2:D9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
jo analysis work in progress
</commit_message>
<xml_diff>
--- a/Documents/DBdesign.xlsx
+++ b/Documents/DBdesign.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF10D9F-43C9-40F4-8D65-AD815682AEAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37AA3DD0-F6FA-4B32-8883-DCF8FAB8608A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="2" xr2:uid="{BEC21941-B947-480A-A7E6-7B63159DE119}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{BEC21941-B947-480A-A7E6-7B63159DE119}"/>
   </bookViews>
   <sheets>
     <sheet name="RBAC+ABAC" sheetId="1" r:id="rId1"/>
     <sheet name="MSForms" sheetId="2" r:id="rId2"/>
     <sheet name="Company Setup" sheetId="3" r:id="rId3"/>
+    <sheet name="Analysis" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="113">
   <si>
     <t>JobOfferUsers</t>
   </si>
@@ -233,9 +234,6 @@
     <t>CandidateApplications</t>
   </si>
   <si>
-    <t>CurrentWorkflowStatusId</t>
-  </si>
-  <si>
     <t>RequestSentDate</t>
   </si>
   <si>
@@ -306,6 +304,72 @@
   </si>
   <si>
     <t>CreatedAt</t>
+  </si>
+  <si>
+    <t>SalaryMatrix</t>
+  </si>
+  <si>
+    <t>SalaryMatrixId</t>
+  </si>
+  <si>
+    <t>WorkFlowStatus</t>
+  </si>
+  <si>
+    <t>WorkFlowName</t>
+  </si>
+  <si>
+    <t>ShortName</t>
+  </si>
+  <si>
+    <t>MatrixName</t>
+  </si>
+  <si>
+    <t>MatrixCode</t>
+  </si>
+  <si>
+    <t>EffectiveFrom</t>
+  </si>
+  <si>
+    <t>EffectiveTo</t>
+  </si>
+  <si>
+    <t>ApprovalStatusId</t>
+  </si>
+  <si>
+    <t>ApprovedByUserId</t>
+  </si>
+  <si>
+    <t>ApprovedAt</t>
+  </si>
+  <si>
+    <t>ModifiedAt</t>
+  </si>
+  <si>
+    <t>ModifiedBy</t>
+  </si>
+  <si>
+    <t>JobOfferWorkFlow</t>
+  </si>
+  <si>
+    <t>CandidateApplicationId</t>
+  </si>
+  <si>
+    <t>WorkFlowStatusId</t>
+  </si>
+  <si>
+    <t>IsDone</t>
+  </si>
+  <si>
+    <t>HiringCompanyId</t>
+  </si>
+  <si>
+    <t>HiringDivisionId</t>
+  </si>
+  <si>
+    <t>JobOfferProposal</t>
+  </si>
+  <si>
+    <t>SalaryMatrixBandId</t>
   </si>
 </sst>
 </file>
@@ -1027,10 +1091,10 @@
         <v>65</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.35">
@@ -1058,7 +1122,7 @@
         <v>16</v>
       </c>
       <c r="H4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.35">
@@ -1066,10 +1130,10 @@
         <v>55</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.35">
@@ -1077,10 +1141,10 @@
         <v>56</v>
       </c>
       <c r="D6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.35">
@@ -1088,10 +1152,10 @@
         <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.35">
@@ -1099,10 +1163,10 @@
         <v>57</v>
       </c>
       <c r="D8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.35">
@@ -1110,10 +1174,10 @@
         <v>58</v>
       </c>
       <c r="D9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.35">
@@ -1121,10 +1185,10 @@
         <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.35">
@@ -1132,10 +1196,10 @@
         <v>60</v>
       </c>
       <c r="D11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.35">
@@ -1143,7 +1207,7 @@
         <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.35">
@@ -1173,11 +1237,185 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AD6FEA5-0945-4178-A2F8-A72772503D4A}">
-  <dimension ref="B2:D9"/>
+  <dimension ref="B2:J18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="21.36328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F4" t="s">
+        <v>94</v>
+      </c>
+      <c r="H4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F5" t="s">
+        <v>95</v>
+      </c>
+      <c r="H5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>109</v>
+      </c>
+      <c r="F6" t="s">
+        <v>50</v>
+      </c>
+      <c r="H6" t="s">
+        <v>96</v>
+      </c>
+      <c r="J6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>110</v>
+      </c>
+      <c r="H7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>75</v>
+      </c>
+      <c r="H9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>89</v>
+      </c>
+      <c r="H10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>90</v>
+      </c>
+      <c r="H11" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="H12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="H13" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="H14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="H15" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="H16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="17" spans="8:8" x14ac:dyDescent="0.35">
+      <c r="H17" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="18" spans="8:8" x14ac:dyDescent="0.35">
+      <c r="H18" t="s">
+        <v>104</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D3A9745-558A-479E-B1B2-9C6EC5EEDA6F}">
+  <dimension ref="B2:D11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="20.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.35">
@@ -1185,7 +1423,7 @@
         <v>66</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
@@ -1201,35 +1439,45 @@
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
-        <v>67</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
-        <v>86</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
-        <v>91</v>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finished jo analysis details page
</commit_message>
<xml_diff>
--- a/Documents/DBdesign.xlsx
+++ b/Documents/DBdesign.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20B1CAE-A912-4902-9064-AE70A491609E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E728A8A2-55D4-4C19-85E5-476B68488387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{BEC21941-B947-480A-A7E6-7B63159DE119}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="155">
   <si>
     <t>JobOfferUsers</t>
   </si>
@@ -451,6 +451,51 @@
   </si>
   <si>
     <t>ItemDescription</t>
+  </si>
+  <si>
+    <t>ValidationStatusId</t>
+  </si>
+  <si>
+    <t>JobOfferAnalysis</t>
+  </si>
+  <si>
+    <t>JobOfferAnalysisId</t>
+  </si>
+  <si>
+    <t>AnalysisNotes</t>
+  </si>
+  <si>
+    <t>RecommendProposalId</t>
+  </si>
+  <si>
+    <t>BestProposalSalary</t>
+  </si>
+  <si>
+    <t>SalaryMatrixBand</t>
+  </si>
+  <si>
+    <t>JobLevelId</t>
+  </si>
+  <si>
+    <t>JobFamilyId</t>
+  </si>
+  <si>
+    <t>PositionGradeId</t>
+  </si>
+  <si>
+    <t>BandMinimum</t>
+  </si>
+  <si>
+    <t>BandMidpoint</t>
+  </si>
+  <si>
+    <t>BandMaximum</t>
+  </si>
+  <si>
+    <t>BelowBandFlagEnabled</t>
+  </si>
+  <si>
+    <t>AboveBandFlagEnabled</t>
   </si>
 </sst>
 </file>
@@ -1509,12 +1554,12 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D3A9745-558A-479E-B1B2-9C6EC5EEDA6F}">
-  <dimension ref="B2:J15"/>
+  <dimension ref="B2:J28"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="20.26953125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.453125" customWidth="1"/>
     <col min="8" max="8" width="23.81640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="25.6328125" bestFit="1" customWidth="1"/>
   </cols>
@@ -1650,9 +1695,6 @@
       </c>
     </row>
     <row r="10" spans="2:10">
-      <c r="B10" t="s">
-        <v>89</v>
-      </c>
       <c r="D10" t="s">
         <v>116</v>
       </c>
@@ -1664,9 +1706,6 @@
       </c>
     </row>
     <row r="11" spans="2:10">
-      <c r="B11" t="s">
-        <v>90</v>
-      </c>
       <c r="D11" t="s">
         <v>117</v>
       </c>
@@ -1682,7 +1721,7 @@
     </row>
     <row r="12" spans="2:10">
       <c r="D12" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F12" t="s">
         <v>1</v>
@@ -1693,7 +1732,7 @@
     </row>
     <row r="13" spans="2:10">
       <c r="D13" t="s">
-        <v>119</v>
+        <v>140</v>
       </c>
       <c r="F13" t="s">
         <v>87</v>
@@ -1704,7 +1743,7 @@
     </row>
     <row r="14" spans="2:10">
       <c r="D14" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="F14" t="s">
         <v>88</v>
@@ -1715,7 +1754,92 @@
     </row>
     <row r="15" spans="2:10">
       <c r="D15" t="s">
-        <v>90</v>
+        <v>142</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4">
+      <c r="B18" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4">
+      <c r="B19" t="s">
+        <v>1</v>
+      </c>
+      <c r="D19" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4">
+      <c r="B20" t="s">
+        <v>92</v>
+      </c>
+      <c r="D20" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4">
+      <c r="B21" t="s">
+        <v>147</v>
+      </c>
+      <c r="D21" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4">
+      <c r="B22" t="s">
+        <v>148</v>
+      </c>
+      <c r="D22" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4">
+      <c r="B23" t="s">
+        <v>149</v>
+      </c>
+      <c r="D23" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4">
+      <c r="B24" t="s">
+        <v>150</v>
+      </c>
+      <c r="D24" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4">
+      <c r="B25" t="s">
+        <v>151</v>
+      </c>
+      <c r="D25" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4">
+      <c r="B26" t="s">
+        <v>152</v>
+      </c>
+      <c r="D26" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4">
+      <c r="B27" t="s">
+        <v>153</v>
+      </c>
+      <c r="D27" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4">
+      <c r="B28" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
salary matriz redesign ui and db table
</commit_message>
<xml_diff>
--- a/Documents/DBdesign.xlsx
+++ b/Documents/DBdesign.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A263095B-ADAD-4812-9CF8-7D5E900CF01A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63ABFC0C-6F04-4EAF-AF7D-CC080DCADF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="7" xr2:uid="{BEC21941-B947-480A-A7E6-7B63159DE119}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="8" xr2:uid="{BEC21941-B947-480A-A7E6-7B63159DE119}"/>
   </bookViews>
   <sheets>
     <sheet name="RBAC+ABAC" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="Discussion" sheetId="6" r:id="rId6"/>
     <sheet name="WorkFlow" sheetId="8" r:id="rId7"/>
     <sheet name="ReDesign" sheetId="9" r:id="rId8"/>
+    <sheet name="Matrix" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="244">
   <si>
     <t>JobOfferUsers</t>
   </si>
@@ -731,6 +732,42 @@
   </si>
   <si>
     <t>ChannelId</t>
+  </si>
+  <si>
+    <t>GradeTypes</t>
+  </si>
+  <si>
+    <t>SalaryGrades</t>
+  </si>
+  <si>
+    <t>GradeName</t>
+  </si>
+  <si>
+    <t>CompanySalaryGrades</t>
+  </si>
+  <si>
+    <t>GradeId</t>
+  </si>
+  <si>
+    <t>SalaryBands</t>
+  </si>
+  <si>
+    <t>CSGId</t>
+  </si>
+  <si>
+    <t>Minimun</t>
+  </si>
+  <si>
+    <t>Midpoint</t>
+  </si>
+  <si>
+    <t>Maximum</t>
+  </si>
+  <si>
+    <t>EffectFrom</t>
+  </si>
+  <si>
+    <t>EffectTo</t>
   </si>
 </sst>
 </file>
@@ -2924,4 +2961,120 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F800367-D121-468C-B2BA-C9E3C3CB19BA}">
+  <dimension ref="B2:L8"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="2" max="2" width="12.54296875" customWidth="1"/>
+    <col min="4" max="4" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.453125" customWidth="1"/>
+    <col min="8" max="8" width="20.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12">
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1</v>
+      </c>
+      <c r="L3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12">
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F4" t="s">
+        <v>125</v>
+      </c>
+      <c r="H4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L4" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12">
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" t="s">
+        <v>234</v>
+      </c>
+      <c r="H5" t="s">
+        <v>236</v>
+      </c>
+      <c r="J5" t="s">
+        <v>242</v>
+      </c>
+      <c r="L5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12">
+      <c r="J6" t="s">
+        <v>243</v>
+      </c>
+      <c r="L6" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12">
+      <c r="J7" t="s">
+        <v>30</v>
+      </c>
+      <c r="L7" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12">
+      <c r="L8" t="s">
+        <v>241</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
matrix done, start benefits
</commit_message>
<xml_diff>
--- a/Documents/DBdesign.xlsx
+++ b/Documents/DBdesign.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63ABFC0C-6F04-4EAF-AF7D-CC080DCADF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB5EC828-5E5E-41B9-B2F1-946A454227EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="8" xr2:uid="{BEC21941-B947-480A-A7E6-7B63159DE119}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="9" xr2:uid="{BEC21941-B947-480A-A7E6-7B63159DE119}"/>
   </bookViews>
   <sheets>
     <sheet name="RBAC+ABAC" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="WorkFlow" sheetId="8" r:id="rId7"/>
     <sheet name="ReDesign" sheetId="9" r:id="rId8"/>
     <sheet name="Matrix" sheetId="10" r:id="rId9"/>
+    <sheet name="Comp&amp;Ben" sheetId="11" r:id="rId10"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="311">
   <si>
     <t>JobOfferUsers</t>
   </si>
@@ -764,17 +765,218 @@
     <t>Maximum</t>
   </si>
   <si>
-    <t>EffectFrom</t>
-  </si>
-  <si>
-    <t>EffectTo</t>
+    <t>PlanName</t>
+  </si>
+  <si>
+    <t>AreaName</t>
+  </si>
+  <si>
+    <t>AreaId</t>
+  </si>
+  <si>
+    <t>ShiftName</t>
+  </si>
+  <si>
+    <t>ShiftId</t>
+  </si>
+  <si>
+    <t>Motorized</t>
+  </si>
+  <si>
+    <t>AllowSpec</t>
+  </si>
+  <si>
+    <t>AllowTrans</t>
+  </si>
+  <si>
+    <t>Incentive</t>
+  </si>
+  <si>
+    <t>NonSwipe</t>
+  </si>
+  <si>
+    <t>PlanId</t>
+  </si>
+  <si>
+    <t>CompBenEmpType</t>
+  </si>
+  <si>
+    <t>CompBenPlans</t>
+  </si>
+  <si>
+    <t>CompBenArea</t>
+  </si>
+  <si>
+    <t>CompBenSched</t>
+  </si>
+  <si>
+    <t>CompBenShift</t>
+  </si>
+  <si>
+    <t>CompBenFreq</t>
+  </si>
+  <si>
+    <t>FreqName</t>
+  </si>
+  <si>
+    <t>CompBenItmCat</t>
+  </si>
+  <si>
+    <t>CatName</t>
+  </si>
+  <si>
+    <t>CatId</t>
+  </si>
+  <si>
+    <t>FreqId</t>
+  </si>
+  <si>
+    <t>ItmName</t>
+  </si>
+  <si>
+    <t>ItmDesc</t>
+  </si>
+  <si>
+    <t>SchedName</t>
+  </si>
+  <si>
+    <t>SchedId</t>
+  </si>
+  <si>
+    <t>Office Based Position</t>
+  </si>
+  <si>
+    <t>Emp Status</t>
+  </si>
+  <si>
+    <t>Probationary</t>
+  </si>
+  <si>
+    <t>Work Area</t>
+  </si>
+  <si>
+    <t>Office</t>
+  </si>
+  <si>
+    <t>Shift Code</t>
+  </si>
+  <si>
+    <t>O11 - 7:30 – 17:30</t>
+  </si>
+  <si>
+    <t>Work Schedule</t>
+  </si>
+  <si>
+    <t>Compressed</t>
+  </si>
+  <si>
+    <t>Swiping Status</t>
+  </si>
+  <si>
+    <t>Swiping</t>
+  </si>
+  <si>
+    <t>Job Class</t>
+  </si>
+  <si>
+    <t>Rank &amp; File</t>
+  </si>
+  <si>
+    <t>MRI</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Transpo Allowance</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Frequency</t>
+  </si>
+  <si>
+    <t>Monthly15</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Incentivized</t>
+  </si>
+  <si>
+    <t>Annual Bonus</t>
+  </si>
+  <si>
+    <t>Special Allowance</t>
+  </si>
+  <si>
+    <t>Salary Grade</t>
+  </si>
+  <si>
+    <t>SG 07*</t>
+  </si>
+  <si>
+    <t>Territory Rep, GMA</t>
+  </si>
+  <si>
+    <t>Field GMA</t>
+  </si>
+  <si>
+    <t>NPO</t>
+  </si>
+  <si>
+    <t>Non-Swiping</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No </t>
+  </si>
+  <si>
+    <t>SG 08</t>
+  </si>
+  <si>
+    <t>Project Employee - Office</t>
+  </si>
+  <si>
+    <t>Temp Project Hire</t>
+  </si>
+  <si>
+    <t>O11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonRegular </t>
+  </si>
+  <si>
+    <t>Monthly13</t>
+  </si>
+  <si>
+    <t>NR</t>
+  </si>
+  <si>
+    <t>CompBenClass</t>
+  </si>
+  <si>
+    <t>ClassName</t>
+  </si>
+  <si>
+    <t>ClassId</t>
+  </si>
+  <si>
+    <t>CompBenMri</t>
+  </si>
+  <si>
+    <t>MriName</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -801,16 +1003,35 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -818,17 +1039,82 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1488,6 +1774,498 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54F2E5B3-A5D7-48E1-BBB6-A4B5E81A5574}">
+  <dimension ref="B1:R33"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="2" max="2" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.1796875" customWidth="1"/>
+    <col min="6" max="6" width="14.26953125" customWidth="1"/>
+    <col min="8" max="8" width="14.6328125" customWidth="1"/>
+    <col min="10" max="10" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:18" ht="15" thickBot="1"/>
+    <row r="2" spans="2:18" ht="15" thickBot="1">
+      <c r="B2" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="L2" s="7"/>
+      <c r="N2" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="O2" s="7"/>
+      <c r="Q2" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="R2" s="7"/>
+    </row>
+    <row r="3" spans="2:18" ht="15" thickBot="1">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="4" spans="2:18" ht="15" thickBot="1">
+      <c r="B4" t="s">
+        <v>242</v>
+      </c>
+      <c r="D4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F4" t="s">
+        <v>252</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="Q4" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="5" spans="2:18" ht="15" thickBot="1">
+      <c r="B5" t="s">
+        <v>125</v>
+      </c>
+      <c r="F5" t="s">
+        <v>262</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="Q5" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="6" spans="2:18" ht="15" thickBot="1">
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>263</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="Q6" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="7" spans="2:18" ht="15" thickBot="1">
+      <c r="B7" t="s">
+        <v>244</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="F7" t="s">
+        <v>264</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="R7" s="5" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="8" spans="2:18" ht="15" thickBot="1">
+      <c r="B8" t="s">
+        <v>267</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s">
+        <v>265</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="R8" s="5" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="9" spans="2:18" ht="15" thickBot="1">
+      <c r="B9" t="s">
+        <v>246</v>
+      </c>
+      <c r="D9" t="s">
+        <v>243</v>
+      </c>
+      <c r="F9" t="s">
+        <v>123</v>
+      </c>
+      <c r="H9" t="s">
+        <v>1</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="N9" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="O9" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="Q9" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="R9" s="5" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="10" spans="2:18" ht="15" thickBot="1">
+      <c r="B10" t="s">
+        <v>247</v>
+      </c>
+      <c r="H10" t="s">
+        <v>261</v>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="N10" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="O10" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="Q10" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="R10" s="5" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="11" spans="2:18" ht="15" thickBot="1">
+      <c r="B11" t="s">
+        <v>249</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="L11" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="N11" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="O11" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="Q11" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="R11" s="5" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="12" spans="2:18" ht="15" thickBot="1">
+      <c r="B12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="L12" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="N12" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="O12" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="Q12" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="R12" s="5" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="13" spans="2:18" ht="15" thickBot="1">
+      <c r="B13" t="s">
+        <v>250</v>
+      </c>
+      <c r="D13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="L13" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="N13" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="O13" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="Q13" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="R13" s="5" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="14" spans="2:18" ht="15" thickBot="1">
+      <c r="B14" t="s">
+        <v>204</v>
+      </c>
+      <c r="D14" t="s">
+        <v>266</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="L14" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="N14" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="O14" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="Q14" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="R14" s="5" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="15" spans="2:18" ht="15" thickBot="1">
+      <c r="B15" t="s">
+        <v>251</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="L15" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="N15" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="O15" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="Q15" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="R15" s="5" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="16" spans="2:18" ht="15" thickBot="1">
+      <c r="B16" t="s">
+        <v>308</v>
+      </c>
+      <c r="K16" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="N16" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="O16" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="Q16" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="R16" s="5" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4">
+      <c r="B17" t="s">
+        <v>238</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4">
+      <c r="D18" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4">
+      <c r="D19" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4">
+      <c r="D22" s="1" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4">
+      <c r="D23" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4">
+      <c r="D24" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4">
+      <c r="D26" s="1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4">
+      <c r="D27" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4">
+      <c r="D28" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4">
+      <c r="D31" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="32" spans="2:4">
+      <c r="D32" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="4:4">
+      <c r="D33" t="s">
+        <v>310</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="Q2:R2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{026B99F0-FC57-47AB-AF03-F4ABCCD02BF2}">
   <dimension ref="B2:H16"/>
@@ -3047,24 +3825,18 @@
         <v>236</v>
       </c>
       <c r="J5" t="s">
-        <v>242</v>
+        <v>30</v>
       </c>
       <c r="L5" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="6" spans="2:12">
-      <c r="J6" t="s">
-        <v>243</v>
-      </c>
       <c r="L6" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="7" spans="2:12">
-      <c r="J7" t="s">
-        <v>30</v>
-      </c>
       <c r="L7" t="s">
         <v>240</v>
       </c>

</xml_diff>

<commit_message>
centralize css themes and design
</commit_message>
<xml_diff>
--- a/Documents/DBdesign.xlsx
+++ b/Documents/DBdesign.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB5EC828-5E5E-41B9-B2F1-946A454227EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A317693D-7169-4E67-902E-1930A0B022A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="9" xr2:uid="{BEC21941-B947-480A-A7E6-7B63159DE119}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="9" xr2:uid="{BEC21941-B947-480A-A7E6-7B63159DE119}"/>
   </bookViews>
   <sheets>
     <sheet name="RBAC+ABAC" sheetId="1" r:id="rId1"/>
@@ -24,10 +24,21 @@
     <sheet name="Matrix" sheetId="10" r:id="rId9"/>
     <sheet name="Comp&amp;Ben" sheetId="11" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
@@ -37,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="310">
   <si>
     <t>JobOfferUsers</t>
   </si>
@@ -826,9 +837,6 @@
   </si>
   <si>
     <t>CatId</t>
-  </si>
-  <si>
-    <t>FreqId</t>
   </si>
   <si>
     <t>ItmName</t>
@@ -1017,7 +1025,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1027,6 +1035,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1093,7 +1107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1108,13 +1122,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1779,7 +1796,7 @@
   <dimension ref="B1:R33"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.1796875" customWidth="1"/>
     <col min="6" max="6" width="14.26953125" customWidth="1"/>
     <col min="8" max="8" width="14.6328125" customWidth="1"/>
@@ -1803,18 +1820,21 @@
       <c r="F2" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="K2" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="L2" s="7"/>
-      <c r="N2" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="O2" s="7"/>
-      <c r="Q2" s="6" t="s">
-        <v>300</v>
-      </c>
-      <c r="R2" s="7"/>
+      <c r="H2" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="L2" s="8"/>
+      <c r="N2" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="O2" s="8"/>
+      <c r="Q2" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="R2" s="8"/>
     </row>
     <row r="3" spans="2:18" ht="15" thickBot="1">
       <c r="B3" t="s">
@@ -1826,23 +1846,26 @@
       <c r="F3" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="H3" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="L3" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="L3" s="5" t="s">
-        <v>270</v>
-      </c>
       <c r="N3" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="O3" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="O3" s="5" t="s">
-        <v>270</v>
-      </c>
       <c r="Q3" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" spans="2:18" ht="15" thickBot="1">
@@ -1855,23 +1878,26 @@
       <c r="F4" t="s">
         <v>252</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="H4" t="s">
+        <v>261</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="L4" s="5" t="s">
-        <v>272</v>
-      </c>
       <c r="N4" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="Q4" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="R4" s="5" t="s">
         <v>271</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>294</v>
-      </c>
-      <c r="Q4" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="R4" s="5" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="5" spans="2:18" ht="15" thickBot="1">
@@ -1881,23 +1907,23 @@
       <c r="F5" t="s">
         <v>262</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="K5" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="L5" s="5" t="s">
         <v>273</v>
       </c>
-      <c r="L5" s="5" t="s">
-        <v>274</v>
-      </c>
       <c r="N5" s="4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="R5" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="6" spans="2:18" ht="15" thickBot="1">
@@ -1907,23 +1933,23 @@
       <c r="F6" t="s">
         <v>263</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="K6" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="L6" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="L6" s="5" t="s">
-        <v>276</v>
-      </c>
       <c r="N6" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="O6" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="O6" s="5" t="s">
-        <v>276</v>
-      </c>
       <c r="Q6" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="R6" s="5" t="s">
         <v>275</v>
-      </c>
-      <c r="R6" s="5" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="7" spans="2:18" ht="15" thickBot="1">
@@ -1936,55 +1962,52 @@
       <c r="F7" t="s">
         <v>264</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="K7" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="L7" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="L7" s="5" t="s">
-        <v>278</v>
-      </c>
       <c r="N7" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="R7" s="5" t="s">
         <v>277</v>
-      </c>
-      <c r="O7" s="5" t="s">
-        <v>296</v>
-      </c>
-      <c r="Q7" s="4" t="s">
-        <v>277</v>
-      </c>
-      <c r="R7" s="5" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="8" spans="2:18" ht="15" thickBot="1">
       <c r="B8" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D8" t="s">
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>265</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="K8" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="L8" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="L8" s="5" t="s">
-        <v>280</v>
-      </c>
       <c r="N8" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="O8" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="O8" s="5" t="s">
-        <v>280</v>
-      </c>
       <c r="Q8" s="4" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="R8" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="9" spans="2:18" ht="15" thickBot="1">
@@ -1995,77 +2018,71 @@
         <v>243</v>
       </c>
       <c r="F9" t="s">
-        <v>123</v>
-      </c>
-      <c r="H9" t="s">
-        <v>1</v>
-      </c>
-      <c r="K9" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="L9" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="L9" s="5" t="s">
-        <v>282</v>
-      </c>
       <c r="N9" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="O9" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="O9" s="5" t="s">
-        <v>282</v>
-      </c>
       <c r="Q9" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="R9" s="5" t="s">
         <v>281</v>
-      </c>
-      <c r="R9" s="5" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="10" spans="2:18" ht="15" thickBot="1">
       <c r="B10" t="s">
         <v>247</v>
       </c>
-      <c r="H10" t="s">
-        <v>261</v>
-      </c>
-      <c r="K10" s="8" t="s">
+      <c r="K10" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="L10" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="L10" s="5" t="s">
-        <v>284</v>
-      </c>
       <c r="N10" s="4" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="Q10" s="4" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="R10" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="11" spans="2:18" ht="15" thickBot="1">
       <c r="B11" t="s">
         <v>249</v>
       </c>
-      <c r="K11" s="8" t="s">
+      <c r="K11" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L11" s="5" t="s">
         <v>285</v>
       </c>
-      <c r="L11" s="5" t="s">
-        <v>286</v>
-      </c>
       <c r="N11" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="O11" s="5" t="s">
         <v>285</v>
       </c>
-      <c r="O11" s="5" t="s">
-        <v>286</v>
-      </c>
       <c r="Q11" s="4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="R11" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="12" spans="2:18" ht="15" thickBot="1">
@@ -2075,23 +2092,23 @@
       <c r="D12" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="K12" s="8" t="s">
+      <c r="K12" s="6" t="s">
         <v>247</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="N12" s="4" t="s">
         <v>247</v>
       </c>
       <c r="O12" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q12" s="4" t="s">
         <v>247</v>
       </c>
       <c r="R12" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="13" spans="2:18" ht="15" thickBot="1">
@@ -2101,23 +2118,23 @@
       <c r="D13" t="s">
         <v>1</v>
       </c>
-      <c r="K13" s="8" t="s">
-        <v>288</v>
+      <c r="K13" s="6" t="s">
+        <v>287</v>
       </c>
       <c r="L13" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="N13" s="4" t="s">
         <v>287</v>
       </c>
-      <c r="N13" s="4" t="s">
-        <v>288</v>
-      </c>
       <c r="O13" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q13" s="4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="R13" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="14" spans="2:18" ht="15" thickBot="1">
@@ -2125,71 +2142,71 @@
         <v>204</v>
       </c>
       <c r="D14" t="s">
-        <v>266</v>
-      </c>
-      <c r="K14" s="8" t="s">
-        <v>289</v>
+        <v>265</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>288</v>
       </c>
       <c r="L14" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="O14" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="Q14" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="R14" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="15" spans="2:18" ht="15" thickBot="1">
       <c r="B15" t="s">
         <v>251</v>
       </c>
-      <c r="K15" s="8" t="s">
-        <v>290</v>
+      <c r="K15" s="6" t="s">
+        <v>289</v>
       </c>
       <c r="L15" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="N15" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="Q15" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="R15" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="16" spans="2:18" ht="15" thickBot="1">
       <c r="B16" t="s">
-        <v>308</v>
-      </c>
-      <c r="K16" s="8" t="s">
+        <v>307</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="L16" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="L16" s="5" t="s">
-        <v>292</v>
-      </c>
       <c r="N16" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="Q16" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="R16" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="17" spans="2:4">
@@ -2210,19 +2227,35 @@
         <v>245</v>
       </c>
     </row>
+    <row r="20" spans="2:4">
+      <c r="B20" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4">
+      <c r="B21" t="s">
+        <v>1</v>
+      </c>
+    </row>
     <row r="22" spans="2:4">
+      <c r="B22" t="s">
+        <v>252</v>
+      </c>
       <c r="D22" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="23" spans="2:4">
+      <c r="B23" t="s">
+        <v>8</v>
+      </c>
       <c r="D23" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="2:4">
       <c r="D24" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="26" spans="2:4">
@@ -2242,7 +2275,7 @@
     </row>
     <row r="31" spans="2:4">
       <c r="D31" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="32" spans="2:4">
@@ -2252,7 +2285,7 @@
     </row>
     <row r="33" spans="4:4">
       <c r="D33" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>